<commit_message>
add new infos, fix bugs, optimize performance
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9731764A-2BE7-4C1F-B37E-B5D422BD4393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C472AB0-80F5-4161-8117-4D55F0294BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="490" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3177" uniqueCount="3026">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3228" uniqueCount="3067">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24077,6 +24077,131 @@
   </si>
   <si>
     <t>确认要重新加载地图吗？</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MapObjectList.Index</t>
+  </si>
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>MapObjectList.Type</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>MapObjectList.DisplayName</t>
+  </si>
+  <si>
+    <t>Name (ID)</t>
+  </si>
+  <si>
+    <t>MapObjectList.Coordinate</t>
+  </si>
+  <si>
+    <t>Coordinate</t>
+  </si>
+  <si>
+    <t>MapObjectList.House</t>
+  </si>
+  <si>
+    <t>MapObjectList.Health</t>
+  </si>
+  <si>
+    <t>MapObjectList.Facing</t>
+  </si>
+  <si>
+    <t>MapObjectList.Status</t>
+  </si>
+  <si>
+    <t>MapObjectList.Tag</t>
+  </si>
+  <si>
+    <t>MapObjectList.Type.Infantry</t>
+  </si>
+  <si>
+    <t>MapObjectList.Type.Unit</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>MapObjectList.Type.Aircraft</t>
+  </si>
+  <si>
+    <t>MapObjectList.Type.Building</t>
+  </si>
+  <si>
+    <t>MapObjectList.Refresh</t>
+  </si>
+  <si>
+    <t>MapObjectList.Count</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>TabPages.MapObjectList</t>
+  </si>
+  <si>
+    <t>Map Objects</t>
+  </si>
+  <si>
+    <t>索引</t>
+  </si>
+  <si>
+    <t>类型</t>
+  </si>
+  <si>
+    <t>名称 (ID)</t>
+  </si>
+  <si>
+    <t>坐标</t>
+  </si>
+  <si>
+    <t>所属方</t>
+  </si>
+  <si>
+    <t>强度</t>
+  </si>
+  <si>
+    <t>面向</t>
+  </si>
+  <si>
+    <t>状态</t>
+  </si>
+  <si>
+    <t>标签</t>
+  </si>
+  <si>
+    <t>步兵</t>
+  </si>
+  <si>
+    <t>车辆</t>
+  </si>
+  <si>
+    <t>飞行器</t>
+  </si>
+  <si>
+    <t>建筑</t>
+  </si>
+  <si>
+    <t>刷新</t>
+  </si>
+  <si>
+    <t>计数</t>
+  </si>
+  <si>
+    <t>地图单位</t>
+  </si>
+  <si>
+    <t>MapObjectList.Search</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>搜索：</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -24480,7 +24605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1061"/>
+  <dimension ref="A1:D1078"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36153,6 +36278,193 @@
         <v>3023</v>
       </c>
     </row>
+    <row r="1062" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1062" s="3" t="s">
+        <v>3026</v>
+      </c>
+      <c r="B1062" s="4" t="s">
+        <v>3049</v>
+      </c>
+      <c r="C1062" s="3" t="s">
+        <v>3027</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1063" s="3" t="s">
+        <v>3028</v>
+      </c>
+      <c r="B1063" s="4" t="s">
+        <v>3050</v>
+      </c>
+      <c r="C1063" s="3" t="s">
+        <v>3029</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1064" s="3" t="s">
+        <v>3030</v>
+      </c>
+      <c r="B1064" s="4" t="s">
+        <v>3051</v>
+      </c>
+      <c r="C1064" s="3" t="s">
+        <v>3031</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1065" s="3" t="s">
+        <v>3032</v>
+      </c>
+      <c r="B1065" s="4" t="s">
+        <v>3052</v>
+      </c>
+      <c r="C1065" s="3" t="s">
+        <v>3033</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1066" s="3" t="s">
+        <v>3034</v>
+      </c>
+      <c r="B1066" s="4" t="s">
+        <v>3053</v>
+      </c>
+      <c r="C1066" s="3" t="s">
+        <v>1228</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1067" s="3" t="s">
+        <v>3035</v>
+      </c>
+      <c r="B1067" s="4" t="s">
+        <v>3054</v>
+      </c>
+      <c r="C1067" s="3" t="s">
+        <v>1671</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1068" s="3" t="s">
+        <v>3036</v>
+      </c>
+      <c r="B1068" s="4" t="s">
+        <v>3055</v>
+      </c>
+      <c r="C1068" s="3" t="s">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1069" s="3" t="s">
+        <v>3037</v>
+      </c>
+      <c r="B1069" s="4" t="s">
+        <v>3056</v>
+      </c>
+      <c r="C1069" s="3" t="s">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1070" s="3" t="s">
+        <v>3038</v>
+      </c>
+      <c r="B1070" s="4" t="s">
+        <v>3057</v>
+      </c>
+      <c r="C1070" s="3" t="s">
+        <v>1689</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1071" s="3" t="s">
+        <v>3039</v>
+      </c>
+      <c r="B1071" s="4" t="s">
+        <v>3058</v>
+      </c>
+      <c r="C1071" s="3" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1072" s="3" t="s">
+        <v>3040</v>
+      </c>
+      <c r="B1072" s="4" t="s">
+        <v>3059</v>
+      </c>
+      <c r="C1072" s="3" t="s">
+        <v>3041</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1073" s="3" t="s">
+        <v>3042</v>
+      </c>
+      <c r="B1073" s="4" t="s">
+        <v>3060</v>
+      </c>
+      <c r="C1073" s="3" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="1074" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1074" s="3" t="s">
+        <v>3043</v>
+      </c>
+      <c r="B1074" s="4" t="s">
+        <v>3061</v>
+      </c>
+      <c r="C1074" s="3" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="1075" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1075" s="3" t="s">
+        <v>3044</v>
+      </c>
+      <c r="B1075" s="4" t="s">
+        <v>3062</v>
+      </c>
+      <c r="C1075" s="3" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="1076" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1076" s="3" t="s">
+        <v>3045</v>
+      </c>
+      <c r="B1076" s="4" t="s">
+        <v>3063</v>
+      </c>
+      <c r="C1076" s="3" t="s">
+        <v>3046</v>
+      </c>
+    </row>
+    <row r="1077" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1077" s="3" t="s">
+        <v>3065</v>
+      </c>
+      <c r="B1077" s="4" t="s">
+        <v>3066</v>
+      </c>
+      <c r="C1077" s="3" t="s">
+        <v>1188</v>
+      </c>
+    </row>
+    <row r="1078" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1078" s="3" t="s">
+        <v>3047</v>
+      </c>
+      <c r="B1078" s="4" t="s">
+        <v>3064</v>
+      </c>
+      <c r="C1078" s="3" t="s">
+        <v>3048</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add ExtTilts to support tilt image on ramps
just a baseline implementation
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C472AB0-80F5-4161-8117-4D55F0294BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45C6D55-E8AF-4139-AD1F-9FC5B0AE16F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="490" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3228" uniqueCount="3067">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3231" uniqueCount="3070">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24203,6 +24203,16 @@
   <si>
     <t>搜索：</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Options.ExtTilts</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Allow vehicles and aircraft to tilt on slopes</t>
+  </si>
+  <si>
+    <t>车辆和飞行器在斜坡上显示倾斜图像</t>
   </si>
 </sst>
 </file>
@@ -24605,7 +24615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1078"/>
+  <dimension ref="A1:D1079"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36465,6 +36475,17 @@
         <v>3048</v>
       </c>
     </row>
+    <row r="1079" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1079" s="3" t="s">
+        <v>3067</v>
+      </c>
+      <c r="B1079" s="4" t="s">
+        <v>3069</v>
+      </c>
+      <c r="C1079" s="3" t="s">
+        <v>3068</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add yolo mode for lua console
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45C6D55-E8AF-4139-AD1F-9FC5B0AE16F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334CD161-581E-49C4-8CDA-AC0A092F7BCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="490" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3231" uniqueCount="3070">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3237" uniqueCount="3076">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24213,6 +24213,27 @@
   </si>
   <si>
     <t>车辆和飞行器在斜坡上显示倾斜图像</t>
+  </si>
+  <si>
+    <t>LuaConsole.YoloModeConfirm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>YOLO mode will skip all confirmation dialogs during script execution.\nThis includes safety checks, snapshot restore confirmations, and building overlap warnings.\nMessage boxes explicitly called by the script (e.g. message_box) will still appear.\n\nAre you sure you want to enable YOLO mode?</t>
+  </si>
+  <si>
+    <t>LuaConsole.YoloModeTitle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Enable YOLO Mode</t>
+  </si>
+  <si>
+    <t>启用YOLO模式</t>
+  </si>
+  <si>
+    <t>YOLO模式将跳过脚本执行期间的所有确认对话框。\n这包括安全检查、快照还原确认和建筑重叠警告。\n由脚本显式调用的对话框（例如message_box）仍将显示。\n\n确定要启用YOLO模式吗？</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -24615,7 +24636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1079"/>
+  <dimension ref="A1:D1081"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36486,6 +36507,28 @@
         <v>3068</v>
       </c>
     </row>
+    <row r="1080" spans="1:3" ht="95" x14ac:dyDescent="0.4">
+      <c r="A1080" s="3" t="s">
+        <v>3070</v>
+      </c>
+      <c r="B1080" s="4" t="s">
+        <v>3075</v>
+      </c>
+      <c r="C1080" s="3" t="s">
+        <v>3071</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1081" s="3" t="s">
+        <v>3072</v>
+      </c>
+      <c r="B1081" s="4" t="s">
+        <v>3074</v>
+      </c>
+      <c r="C1081" s="3" t="s">
+        <v>3073</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add search dialog in object view
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481C053E-83C7-429D-A44C-31ADF4B9614C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08E821D8-1833-4747-8446-3F4BE7683A75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4560" yWindow="3170" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3246" uniqueCount="3085">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3249" uniqueCount="3087">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24123,6 +24123,14 @@
   </si>
   <si>
     <t>Consider sub tile blocks as identical when ctrl-filling areas</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>搜索:</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ViewObjects.SearchLabel</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -24526,7 +24534,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1084"/>
+  <dimension ref="A1:D1085"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36452,6 +36460,17 @@
         <v>3084</v>
       </c>
     </row>
+    <row r="1085" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1085" s="3" t="s">
+        <v>3086</v>
+      </c>
+      <c r="B1085" s="4" t="s">
+        <v>3085</v>
+      </c>
+      <c r="C1085" s="3" t="s">
+        <v>1188</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add phobos v0.5-alpha actions & scripts
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D92D16-1FF3-41E4-AEE3-1ED5203D0E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E78DDD-258B-4C06-A7F6-3713DC37ACE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4560" yWindow="3170" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24119,12 +24119,12 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve"> (Phobos v0.5-aplha+)</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Show &lt;Player @ X&gt; options in trigger editor (Phobos v0.5-aplha+)</t>
+      <t xml:space="preserve"> (Phobos v0.5-alpha+)</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Show &lt;Player @ X&gt; options in trigger editor (Phobos v0.5-alpha+)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>

</xml_diff>

<commit_message>
fix bugs, adjust control positions
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08E821D8-1833-4747-8446-3F4BE7683A75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAF02AA-55C0-40BB-80C1-060BC4BB9283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4560" yWindow="3170" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5120" yWindow="2710" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3249" uniqueCount="3087">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3273" uniqueCount="3112">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24014,123 +24014,307 @@
     <t>所属方</t>
   </si>
   <si>
-    <t>强度</t>
+    <t>状态</t>
+  </si>
+  <si>
+    <t>标签</t>
+  </si>
+  <si>
+    <t>步兵</t>
+  </si>
+  <si>
+    <t>车辆</t>
+  </si>
+  <si>
+    <t>飞行器</t>
+  </si>
+  <si>
+    <t>建筑</t>
+  </si>
+  <si>
+    <t>刷新</t>
+  </si>
+  <si>
+    <t>计数</t>
+  </si>
+  <si>
+    <t>MapObjectList.Search</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>搜索：</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Options.ExtTilts</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Allow vehicles and aircraft to tilt on slopes</t>
+  </si>
+  <si>
+    <t>车辆和飞行器在斜坡上显示倾斜图像</t>
+  </si>
+  <si>
+    <t>LuaConsole.YoloModeConfirm</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>YOLO mode will skip all confirmation dialogs during script execution.\nThis includes safety checks, snapshot restore confirmations, and building overlap warnings.\nMessage boxes explicitly called by the script (e.g. message_box) will still appear.\n\nAre you sure you want to enable YOLO mode?</t>
+  </si>
+  <si>
+    <t>LuaConsole.YoloModeTitle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Enable YOLO Mode</t>
+  </si>
+  <si>
+    <t>启用YOLO模式</t>
+  </si>
+  <si>
+    <t>YOLO模式将跳过脚本执行期间的所有确认对话框。\n这包括安全检查、快照还原确认和建筑重叠警告。\n由脚本显式调用的对话框（例如message_box）仍将显示。\n\n确定要启用YOLO模式吗？</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LuaScriptConsoleReset</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reset Lua</t>
+  </si>
+  <si>
+    <t>重置Lua</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Check 'Run File' to read the selected Lua script. Otherwise, the input window will be used. Click 'Run' to run the selected code. Click 'Lua Brush' to run the script at the specified coordinates on the map. Click 'Reset Lua' to reset Lua state. Scripts may damage the map, please save it or execute the snapshot function before running. Please refer to the documentation for available functions.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>勾选“执行文件”以读取选中的Lua脚本，否则读取输入窗口。点击“执行”以执行所选的代码。点击“脚本刷”在地图的指定坐标执行脚本。点击“重置Lua”以清除Lua状态。脚本可能会损坏地图，请在运行前保存或执行快照函数。请参阅文档了解可用函数。</t>
+  </si>
+  <si>
+    <t>Options.UnifyHouseColors</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>将单位所属色变体映射为纯色</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Map house color variants to their corresponding solid colors</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Options.FillArea.ConsiderWholeTile</t>
+  </si>
+  <si>
+    <t>ctrl填充地形时将整个地形的子地形块视作一类</t>
+  </si>
+  <si>
+    <t>Consider sub tile blocks as identical when ctrl-filling areas</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>搜索:</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ViewObjects.SearchLabel</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>地图单位列表</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>面向</t>
-  </si>
-  <si>
-    <t>状态</t>
-  </si>
-  <si>
-    <t>标签</t>
-  </si>
-  <si>
-    <t>步兵</t>
-  </si>
-  <si>
-    <t>车辆</t>
-  </si>
-  <si>
-    <t>飞行器</t>
-  </si>
-  <si>
-    <t>建筑</t>
-  </si>
-  <si>
-    <t>刷新</t>
-  </si>
-  <si>
-    <t>计数</t>
-  </si>
-  <si>
-    <t>地图单位</t>
-  </si>
-  <si>
-    <t>MapObjectList.Search</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>搜索：</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Options.ExtTilts</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Allow vehicles and aircraft to tilt on slopes</t>
-  </si>
-  <si>
-    <t>车辆和飞行器在斜坡上显示倾斜图像</t>
-  </si>
-  <si>
-    <t>LuaConsole.YoloModeConfirm</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>YOLO mode will skip all confirmation dialogs during script execution.\nThis includes safety checks, snapshot restore confirmations, and building overlap warnings.\nMessage boxes explicitly called by the script (e.g. message_box) will still appear.\n\nAre you sure you want to enable YOLO mode?</t>
-  </si>
-  <si>
-    <t>LuaConsole.YoloModeTitle</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Enable YOLO Mode</t>
-  </si>
-  <si>
-    <t>启用YOLO模式</t>
-  </si>
-  <si>
-    <t>YOLO模式将跳过脚本执行期间的所有确认对话框。\n这包括安全检查、快照还原确认和建筑重叠警告。\n由脚本显式调用的对话框（例如message_box）仍将显示。\n\n确定要启用YOLO模式吗？</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>LuaScriptConsoleReset</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Reset Lua</t>
-  </si>
-  <si>
-    <t>重置Lua</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Check 'Run File' to read the selected Lua script. Otherwise, the input window will be used. Click 'Run' to run the selected code. Click 'Lua Brush' to run the script at the specified coordinates on the map. Click 'Reset Lua' to reset Lua state. Scripts may damage the map, please save it or execute the snapshot function before running. Please refer to the documentation for available functions.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>勾选“执行文件”以读取选中的Lua脚本，否则读取输入窗口。点击“执行”以执行所选的代码。点击“脚本刷”在地图的指定坐标执行脚本。点击“重置Lua”以清除Lua状态。脚本可能会损坏地图，请在运行前保存或执行快照函数。请参阅文档了解可用函数。</t>
-  </si>
-  <si>
-    <t>Options.UnifyHouseColors</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>将单位所属色变体映射为纯色</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Map house color variants to their corresponding solid colors</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Options.FillArea.ConsiderWholeTile</t>
-  </si>
-  <si>
-    <t>ctrl填充地形时将整个地形的子地形块视作一类</t>
-  </si>
-  <si>
-    <t>Consider sub tile blocks as identical when ctrl-filling areas</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>搜索:</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>ViewObjects.SearchLabel</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>↗ 东北</t>
+  </si>
+  <si>
+    <t>→ 东</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>↘ 东南</t>
+  </si>
+  <si>
+    <t>↓ 南</t>
+  </si>
+  <si>
+    <t>↙ 西南</t>
+  </si>
+  <si>
+    <t>← 西</t>
+  </si>
+  <si>
+    <t>↖ 西北</t>
+  </si>
+  <si>
+    <t>↑ 北</t>
+  </si>
+  <si>
+    <t>Direction.North</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Direction.NorthWest</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Direction.West</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Direction.SouthWest</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Direction.South</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Direction.SouthEast</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Direction.East</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Direction.NorthEast</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> East</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>←</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> West</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="3"/>
+      </rPr>
+      <t>↗</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> North-East</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="3"/>
+      </rPr>
+      <t>↘</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> South-East</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>↓ South</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="3"/>
+      </rPr>
+      <t>↙</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> South-West</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="3"/>
+      </rPr>
+      <t>↖</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> North-West</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>↑ North</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Health (%)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>生命值 (%)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -24138,7 +24322,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -24205,6 +24389,18 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Segoe UI Symbol"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -24238,7 +24434,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -24253,6 +24449,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="标题 1" xfId="1" builtinId="16"/>
@@ -24534,7 +24733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1085"/>
+  <dimension ref="A1:D1093"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -31196,10 +31395,10 @@
         <v>573</v>
       </c>
       <c r="B607" s="4" t="s">
-        <v>3078</v>
+        <v>3075</v>
       </c>
       <c r="C607" s="3" t="s">
-        <v>3077</v>
+        <v>3074</v>
       </c>
     </row>
     <row r="608" spans="1:3" x14ac:dyDescent="0.4">
@@ -36267,10 +36466,10 @@
         <v>3033</v>
       </c>
       <c r="B1067" s="4" t="s">
-        <v>3052</v>
+        <v>3111</v>
       </c>
       <c r="C1067" s="3" t="s">
-        <v>1670</v>
+        <v>3110</v>
       </c>
     </row>
     <row r="1068" spans="1:3" x14ac:dyDescent="0.4">
@@ -36278,7 +36477,7 @@
         <v>3034</v>
       </c>
       <c r="B1068" s="4" t="s">
-        <v>3053</v>
+        <v>3085</v>
       </c>
       <c r="C1068" s="3" t="s">
         <v>1672</v>
@@ -36289,7 +36488,7 @@
         <v>3035</v>
       </c>
       <c r="B1069" s="4" t="s">
-        <v>3054</v>
+        <v>3052</v>
       </c>
       <c r="C1069" s="3" t="s">
         <v>1689</v>
@@ -36300,7 +36499,7 @@
         <v>3036</v>
       </c>
       <c r="B1070" s="4" t="s">
-        <v>3055</v>
+        <v>3053</v>
       </c>
       <c r="C1070" s="3" t="s">
         <v>1688</v>
@@ -36311,7 +36510,7 @@
         <v>3037</v>
       </c>
       <c r="B1071" s="4" t="s">
-        <v>3056</v>
+        <v>3054</v>
       </c>
       <c r="C1071" s="3" t="s">
         <v>1009</v>
@@ -36322,7 +36521,7 @@
         <v>3038</v>
       </c>
       <c r="B1072" s="4" t="s">
-        <v>3057</v>
+        <v>3055</v>
       </c>
       <c r="C1072" s="3" t="s">
         <v>3039</v>
@@ -36333,7 +36532,7 @@
         <v>3040</v>
       </c>
       <c r="B1073" s="4" t="s">
-        <v>3058</v>
+        <v>3056</v>
       </c>
       <c r="C1073" s="3" t="s">
         <v>1008</v>
@@ -36344,7 +36543,7 @@
         <v>3041</v>
       </c>
       <c r="B1074" s="4" t="s">
-        <v>3059</v>
+        <v>3057</v>
       </c>
       <c r="C1074" s="3" t="s">
         <v>903</v>
@@ -36355,7 +36554,7 @@
         <v>3042</v>
       </c>
       <c r="B1075" s="4" t="s">
-        <v>3060</v>
+        <v>3058</v>
       </c>
       <c r="C1075" s="3" t="s">
         <v>998</v>
@@ -36366,7 +36565,7 @@
         <v>3043</v>
       </c>
       <c r="B1076" s="4" t="s">
-        <v>3061</v>
+        <v>3059</v>
       </c>
       <c r="C1076" s="3" t="s">
         <v>3044</v>
@@ -36374,10 +36573,10 @@
     </row>
     <row r="1077" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1077" s="3" t="s">
-        <v>3063</v>
+        <v>3060</v>
       </c>
       <c r="B1077" s="4" t="s">
-        <v>3064</v>
+        <v>3061</v>
       </c>
       <c r="C1077" s="3" t="s">
         <v>1188</v>
@@ -36388,7 +36587,7 @@
         <v>3045</v>
       </c>
       <c r="B1078" s="4" t="s">
-        <v>3062</v>
+        <v>3084</v>
       </c>
       <c r="C1078" s="3" t="s">
         <v>3046</v>
@@ -36396,79 +36595,167 @@
     </row>
     <row r="1079" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1079" s="3" t="s">
-        <v>3065</v>
+        <v>3062</v>
       </c>
       <c r="B1079" s="4" t="s">
-        <v>3067</v>
+        <v>3064</v>
       </c>
       <c r="C1079" s="3" t="s">
-        <v>3066</v>
+        <v>3063</v>
       </c>
     </row>
     <row r="1080" spans="1:3" ht="95" x14ac:dyDescent="0.4">
       <c r="A1080" s="3" t="s">
-        <v>3068</v>
+        <v>3065</v>
       </c>
       <c r="B1080" s="4" t="s">
-        <v>3073</v>
+        <v>3070</v>
       </c>
       <c r="C1080" s="3" t="s">
-        <v>3069</v>
+        <v>3066</v>
       </c>
     </row>
     <row r="1081" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1081" s="3" t="s">
-        <v>3070</v>
+        <v>3067</v>
       </c>
       <c r="B1081" s="4" t="s">
-        <v>3072</v>
+        <v>3069</v>
       </c>
       <c r="C1081" s="3" t="s">
-        <v>3071</v>
+        <v>3068</v>
       </c>
     </row>
     <row r="1082" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1082" s="3" t="s">
-        <v>3074</v>
+        <v>3071</v>
       </c>
       <c r="B1082" s="4" t="s">
-        <v>3076</v>
+        <v>3073</v>
       </c>
       <c r="C1082" s="3" t="s">
-        <v>3075</v>
+        <v>3072</v>
       </c>
     </row>
     <row r="1083" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1083" s="3" t="s">
-        <v>3079</v>
+        <v>3076</v>
       </c>
       <c r="B1083" s="4" t="s">
-        <v>3080</v>
+        <v>3077</v>
       </c>
       <c r="C1083" s="3" t="s">
-        <v>3081</v>
+        <v>3078</v>
       </c>
     </row>
     <row r="1084" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1084" s="3" t="s">
-        <v>3082</v>
+        <v>3079</v>
       </c>
       <c r="B1084" s="4" t="s">
-        <v>3083</v>
+        <v>3080</v>
       </c>
       <c r="C1084" s="3" t="s">
-        <v>3084</v>
+        <v>3081</v>
       </c>
     </row>
     <row r="1085" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1085" s="3" t="s">
-        <v>3086</v>
+        <v>3083</v>
       </c>
       <c r="B1085" s="4" t="s">
-        <v>3085</v>
+        <v>3082</v>
       </c>
       <c r="C1085" s="3" t="s">
         <v>1188</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:3" ht="22.5" x14ac:dyDescent="0.6">
+      <c r="A1086" s="3" t="s">
+        <v>3101</v>
+      </c>
+      <c r="B1086" s="4" t="s">
+        <v>3086</v>
+      </c>
+      <c r="C1086" s="6" t="s">
+        <v>3104</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1087" s="3" t="s">
+        <v>3100</v>
+      </c>
+      <c r="B1087" s="4" t="s">
+        <v>3087</v>
+      </c>
+      <c r="C1087" s="4" t="s">
+        <v>3102</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:3" ht="22.5" x14ac:dyDescent="0.6">
+      <c r="A1088" s="3" t="s">
+        <v>3099</v>
+      </c>
+      <c r="B1088" s="4" t="s">
+        <v>3088</v>
+      </c>
+      <c r="C1088" s="6" t="s">
+        <v>3105</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1089" s="3" t="s">
+        <v>3098</v>
+      </c>
+      <c r="B1089" s="4" t="s">
+        <v>3089</v>
+      </c>
+      <c r="C1089" s="3" t="s">
+        <v>3106</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:3" ht="22.5" x14ac:dyDescent="0.6">
+      <c r="A1090" s="3" t="s">
+        <v>3097</v>
+      </c>
+      <c r="B1090" s="4" t="s">
+        <v>3090</v>
+      </c>
+      <c r="C1090" s="6" t="s">
+        <v>3107</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1091" s="3" t="s">
+        <v>3096</v>
+      </c>
+      <c r="B1091" s="4" t="s">
+        <v>3091</v>
+      </c>
+      <c r="C1091" s="4" t="s">
+        <v>3103</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:3" ht="22.5" x14ac:dyDescent="0.6">
+      <c r="A1092" s="3" t="s">
+        <v>3095</v>
+      </c>
+      <c r="B1092" s="4" t="s">
+        <v>3092</v>
+      </c>
+      <c r="C1092" s="6" t="s">
+        <v>3108</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1093" s="3" t="s">
+        <v>3094</v>
+      </c>
+      <c r="B1093" s="4" t="s">
+        <v>3093</v>
+      </c>
+      <c r="C1093" s="3" t="s">
+        <v>3109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>